<commit_message>
Verify Emblem vs TMG tax engines; add apples-to-apples 2031 tax block to workbook
</commit_message>
<xml_diff>
--- a/knowledge/exhibits/Boise_Deals_Normalized_Underwriting_v2.xlsx
+++ b/knowledge/exhibits/Boise_Deals_Normalized_Underwriting_v2.xlsx
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="422" uniqueCount="388">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="439" uniqueCount="403">
   <si>
     <t xml:space="preserve">Boise MSA — Deal Comparison &amp; Developer Underwriting Normalization (v2)</t>
   </si>
@@ -619,7 +619,7 @@
     <t xml:space="preserve">Untrended taxes embedded ($, est)</t>
   </si>
   <si>
-    <t xml:space="preserve">2031 taxes deflated 3%/yr</t>
+    <t xml:space="preserve">2031 taxes deflated 3%/yr; consistent with their cost-basis assessment path (~$73.5M 2026-equiv x 0.45%)</t>
   </si>
   <si>
     <t xml:space="preserve">Sale F12 NOI ($, Jan-30)</t>
@@ -773,6 +773,51 @@
   </si>
   <si>
     <t xml:space="preserve">  @ alt cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">D. TAX METHODOLOGY — VERIFIED, THEIRS vs OURS (apples-to-apples)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">THEIR ENGINE (Tax Calcs tab): assessment = cumulative construction cost; steps to $80.3M at completion (2030), +3%/yr to ~$82.7-85.4M in 2031 = ~83% of their own $102.5M sale. Taxed at 0.45%. Construction-period taxes capitalized (fine). NO step-up to value at stabilization and NO reassessment for the buyer at sale.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OUR ENGINE (Seasons Taxes tab): current assessment $92.99M = 78.8% of our price; reassessment year 2027 steps taxable value to 95% x purchase price ($112.1M); +3.5%/yr assessment, -2%/yr levy; exit F12 NOI trued up to buyer taxes at 95% x EXIT price (= the -$15,345 adj in Assumptions M38).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Emblem 2031 taxes as modeled ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A-OperBgt col H; = $1,501/u; implied assessment $85.4M</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Emblem 2031 NOI-ex-tax ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TMG-convention value @ C34 cap ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">closed-form: V = NOI-ex-tax / (cap + 0.95 x levy)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TMG-convention 2031 taxes ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vs $1,501/u as modeled</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Understatement ($/yr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~8-11bp of stabilized YoC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Capitalized impact on exit value ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">~1.0-1.5% of their gross sale</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SYMMETRY NOTE: Seasons current assessment (79% of price) shows the same assessor lag Emblem banks on — but TMG conservatively steps to 95% within a year on BOTH sides of the trade. If you underwrote Seasons on Emblem-style lag, Y1 taxes would be ~$419K not $482K (+5bp on the Y1 cap). The convention difference, not the levy, is the entire dispute.</t>
   </si>
   <si>
     <t xml:space="preserve">The Judy (Hawkins) — Normalization Detail</t>
@@ -1873,84 +1918,84 @@
   <sheetData>
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>368</v>
+        <v>383</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="34" t="s">
-        <v>369</v>
+        <v>384</v>
       </c>
       <c r="C4" s="35" t="s">
-        <v>370</v>
+        <v>385</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="34" t="s">
-        <v>371</v>
+        <v>386</v>
       </c>
       <c r="C5" s="35" t="s">
-        <v>372</v>
+        <v>387</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="34" t="s">
-        <v>373</v>
+        <v>388</v>
       </c>
       <c r="C6" s="35" t="s">
-        <v>374</v>
+        <v>389</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="34" t="s">
-        <v>375</v>
+        <v>390</v>
       </c>
       <c r="C7" s="35" t="s">
-        <v>376</v>
+        <v>391</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="34" t="s">
-        <v>377</v>
+        <v>392</v>
       </c>
       <c r="C8" s="35" t="s">
-        <v>378</v>
+        <v>393</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="34" t="s">
-        <v>379</v>
+        <v>394</v>
       </c>
       <c r="C9" s="35" t="s">
-        <v>380</v>
+        <v>395</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="34" t="s">
-        <v>381</v>
+        <v>396</v>
       </c>
       <c r="C10" s="35" t="s">
-        <v>382</v>
+        <v>397</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="34" t="s">
-        <v>383</v>
+        <v>398</v>
       </c>
       <c r="C11" s="35" t="s">
-        <v>384</v>
+        <v>399</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="34" t="s">
-        <v>385</v>
+        <v>400</v>
       </c>
       <c r="C12" s="35" t="s">
-        <v>386</v>
+        <v>401</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="29" t="s">
-        <v>387</v>
+        <v>402</v>
       </c>
     </row>
   </sheetData>
@@ -3969,7 +4014,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B2:F51"/>
+  <dimension ref="B2:F68"/>
   <sheetFormatPr defaultColWidth="8.5390625" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="2"/>
@@ -4061,7 +4106,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="13" t="s">
         <v>195</v>
       </c>
@@ -4450,7 +4495,147 @@
       </c>
       <c r="F51" s="2"/>
     </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B54" s="14" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B55" s="16" t="s">
+        <v>249</v>
+      </c>
+      <c r="C55" s="16"/>
+      <c r="D55" s="16"/>
+      <c r="E55" s="16"/>
+      <c r="F55" s="16"/>
+    </row>
+    <row r="56" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B56" s="16" t="s">
+        <v>250</v>
+      </c>
+      <c r="C56" s="16"/>
+      <c r="D56" s="16"/>
+      <c r="E56" s="16"/>
+      <c r="F56" s="16"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B57" s="13" t="s">
+        <v>251</v>
+      </c>
+      <c r="C57" s="9" t="n">
+        <v>384319</v>
+      </c>
+      <c r="F57" s="2" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B58" s="13" t="s">
+        <v>253</v>
+      </c>
+      <c r="C58" s="10" t="n">
+        <f aca="false">5825182+C57</f>
+        <v>6209501</v>
+      </c>
+      <c r="F58" s="2"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B59" s="13" t="s">
+        <v>254</v>
+      </c>
+      <c r="C59" s="10" t="n">
+        <f aca="false">C58/(C34+C33)</f>
+        <v>109370339.057684</v>
+      </c>
+      <c r="F59" s="2" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B60" s="13" t="s">
+        <v>256</v>
+      </c>
+      <c r="C60" s="10" t="n">
+        <f aca="false">C33*C59</f>
+        <v>467558.199471598</v>
+      </c>
+      <c r="F60" s="2"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B61" s="13" t="s">
+        <v>236</v>
+      </c>
+      <c r="C61" s="10" t="n">
+        <f aca="false">C60/C8</f>
+        <v>1826.39921668593</v>
+      </c>
+      <c r="F61" s="2" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B62" s="6" t="s">
+        <v>258</v>
+      </c>
+      <c r="C62" s="10" t="n">
+        <f aca="false">C60-C57</f>
+        <v>83239.1994715983</v>
+      </c>
+      <c r="F62" s="2" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B63" s="6" t="s">
+        <v>260</v>
+      </c>
+      <c r="C63" s="10" t="n">
+        <f aca="false">C62/C34</f>
+        <v>1585508.56136378</v>
+      </c>
+      <c r="F63" s="2" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B64" s="13" t="s">
+        <v>236</v>
+      </c>
+      <c r="C64" s="10" t="n">
+        <f aca="false">C63/C8</f>
+        <v>6193.39281782726</v>
+      </c>
+      <c r="F64" s="2"/>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B66" s="16" t="s">
+        <v>262</v>
+      </c>
+      <c r="C66" s="16"/>
+      <c r="D66" s="16"/>
+      <c r="E66" s="16"/>
+      <c r="F66" s="16"/>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B67" s="16"/>
+      <c r="C67" s="16"/>
+      <c r="D67" s="16"/>
+      <c r="E67" s="16"/>
+      <c r="F67" s="16"/>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B68" s="16"/>
+      <c r="C68" s="16"/>
+      <c r="D68" s="16"/>
+      <c r="E68" s="16"/>
+      <c r="F68" s="16"/>
+    </row>
   </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B55:F55"/>
+    <mergeCell ref="B56:F56"/>
+    <mergeCell ref="B66:F68"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -4477,12 +4662,12 @@
   <sheetData>
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>248</v>
+        <v>263</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="43.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
-        <v>249</v>
+        <v>264</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4528,7 +4713,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="13" t="s">
-        <v>250</v>
+        <v>265</v>
       </c>
       <c r="C10" s="10" t="n">
         <f aca="false">C9*C6</f>
@@ -4538,7 +4723,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="13" t="s">
-        <v>251</v>
+        <v>266</v>
       </c>
       <c r="C11" s="9" t="n">
         <v>2914298</v>
@@ -4547,41 +4732,41 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="13" t="s">
-        <v>252</v>
+        <v>267</v>
       </c>
       <c r="C12" s="9" t="n">
         <v>356965</v>
       </c>
       <c r="F12" s="2" t="s">
-        <v>253</v>
+        <v>268</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="13" t="s">
-        <v>254</v>
+        <v>269</v>
       </c>
       <c r="C13" s="10" t="n">
         <f aca="false">C12/1.03^3</f>
         <v>326673.542431001</v>
       </c>
       <c r="F13" s="2" t="s">
-        <v>255</v>
+        <v>270</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="13" t="s">
-        <v>256</v>
+        <v>271</v>
       </c>
       <c r="C14" s="9" t="n">
         <v>578083</v>
       </c>
       <c r="F14" s="2" t="s">
-        <v>257</v>
+        <v>272</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="13" t="s">
-        <v>258</v>
+        <v>273</v>
       </c>
       <c r="C15" s="9" t="n">
         <v>3075765</v>
@@ -4606,23 +4791,23 @@
         <v>58586000</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>259</v>
+        <v>274</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="13" t="s">
-        <v>260</v>
+        <v>275</v>
       </c>
       <c r="C18" s="9" t="n">
         <v>2448783</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>261</v>
+        <v>276</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="13" t="s">
-        <v>262</v>
+        <v>277</v>
       </c>
       <c r="C19" s="28" t="n">
         <v>6.13</v>
@@ -4631,7 +4816,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="14" t="s">
-        <v>263</v>
+        <v>278</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4642,7 +4827,7 @@
         <v>3000</v>
       </c>
       <c r="F22" s="2" t="s">
-        <v>264</v>
+        <v>279</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4657,13 +4842,13 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="13" t="s">
-        <v>265</v>
+        <v>280</v>
       </c>
       <c r="C24" s="11" t="n">
         <v>0.0092</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>266</v>
+        <v>281</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4687,24 +4872,24 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="13" t="s">
-        <v>267</v>
+        <v>282</v>
       </c>
       <c r="C27" s="27" t="n">
         <v>0.0525</v>
       </c>
       <c r="F27" s="2" t="s">
-        <v>268</v>
+        <v>283</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="13" t="s">
-        <v>269</v>
+        <v>284</v>
       </c>
       <c r="C28" s="26" t="n">
         <v>625000</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>270</v>
+        <v>285</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4714,19 +4899,19 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="13" t="s">
-        <v>271</v>
+        <v>286</v>
       </c>
       <c r="C31" s="10" t="n">
         <f aca="false">C10+C13+C23*0.9413</f>
         <v>2958295.893331</v>
       </c>
       <c r="F31" s="2" t="s">
-        <v>272</v>
+        <v>287</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="13" t="s">
-        <v>273</v>
+        <v>288</v>
       </c>
       <c r="C32" s="10" t="n">
         <f aca="false">C31/(C27+C26)</f>
@@ -4736,7 +4921,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="13" t="s">
-        <v>274</v>
+        <v>289</v>
       </c>
       <c r="C33" s="10" t="n">
         <f aca="false">C26*C32</f>
@@ -4753,7 +4938,7 @@
         <v>2606.17063281815</v>
       </c>
       <c r="F34" s="2" t="s">
-        <v>275</v>
+        <v>290</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4768,14 +4953,14 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="6" t="s">
-        <v>276</v>
+        <v>291</v>
       </c>
       <c r="C36" s="21" t="n">
         <f aca="false">C35/C6</f>
         <v>0.0608297357759334</v>
       </c>
       <c r="F36" s="2" t="s">
-        <v>277</v>
+        <v>292</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4787,12 +4972,12 @@
         <v>3354160.940263</v>
       </c>
       <c r="F37" s="2" t="s">
-        <v>278</v>
+        <v>293</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B38" s="13" t="s">
-        <v>279</v>
+        <v>294</v>
       </c>
       <c r="C38" s="10" t="n">
         <f aca="false">C37/(C27+C26)</f>
@@ -4809,17 +4994,17 @@
         <v>338091.070576703</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>280</v>
+        <v>295</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B40" s="14" t="s">
-        <v>281</v>
+        <v>296</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B41" s="13" t="s">
-        <v>282</v>
+        <v>297</v>
       </c>
       <c r="C41" s="10" t="n">
         <f aca="false">C28*C19</f>
@@ -4829,7 +5014,7 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B42" s="13" t="s">
-        <v>283</v>
+        <v>298</v>
       </c>
       <c r="C42" s="10" t="n">
         <f aca="false">C41-C18</f>
@@ -4839,7 +5024,7 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B43" s="13" t="s">
-        <v>284</v>
+        <v>299</v>
       </c>
       <c r="C43" s="10" t="n">
         <f aca="false">C6+C42</f>
@@ -4849,14 +5034,14 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B44" s="6" t="s">
-        <v>285</v>
+        <v>300</v>
       </c>
       <c r="C44" s="21" t="n">
         <f aca="false">C35/C43</f>
         <v>0.0588774039935301</v>
       </c>
       <c r="F44" s="2" t="s">
-        <v>286</v>
+        <v>301</v>
       </c>
     </row>
   </sheetData>
@@ -4886,22 +5071,22 @@
   <sheetData>
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>287</v>
+        <v>302</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B3" s="2" t="s">
-        <v>288</v>
+        <v>303</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="14" t="s">
-        <v>289</v>
+        <v>304</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="29" t="s">
-        <v>290</v>
+        <v>305</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4946,7 +5131,7 @@
         <v>0.0720729413872807</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>291</v>
+        <v>306</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5051,7 +5236,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="14" t="s">
-        <v>292</v>
+        <v>307</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5096,7 +5281,7 @@
         <v>2.21140419805461</v>
       </c>
       <c r="J17" s="2" t="s">
-        <v>293</v>
+        <v>308</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5226,24 +5411,24 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="14" t="s">
-        <v>294</v>
+        <v>309</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C25" s="7" t="s">
-        <v>295</v>
+        <v>310</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>296</v>
+        <v>311</v>
       </c>
       <c r="E25" s="7" t="s">
-        <v>297</v>
+        <v>312</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>298</v>
+        <v>313</v>
       </c>
       <c r="G25" s="7" t="s">
-        <v>299</v>
+        <v>314</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5271,7 +5456,7 @@
         <v>0.0600840809502929</v>
       </c>
       <c r="J26" s="2" t="s">
-        <v>300</v>
+        <v>315</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5376,7 +5561,7 @@
     </row>
     <row r="33" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="2" t="s">
-        <v>301</v>
+        <v>316</v>
       </c>
     </row>
   </sheetData>
@@ -5406,31 +5591,31 @@
   <sheetData>
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>302</v>
+        <v>317</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="14" t="s">
-        <v>303</v>
+        <v>318</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="5" t="s">
-        <v>304</v>
+        <v>319</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>305</v>
+        <v>320</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>306</v>
+        <v>321</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>307</v>
+        <v>322</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="13" t="s">
-        <v>308</v>
+        <v>323</v>
       </c>
       <c r="C6" s="31" t="n">
         <v>0.004053</v>
@@ -5439,12 +5624,12 @@
         <v>0.002033</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>309</v>
+        <v>324</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="13" t="s">
-        <v>310</v>
+        <v>325</v>
       </c>
       <c r="C7" s="31" t="n">
         <v>0.002797</v>
@@ -5453,12 +5638,12 @@
         <v>0.000332</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>311</v>
+        <v>326</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="13" t="s">
-        <v>312</v>
+        <v>327</v>
       </c>
       <c r="C8" s="31" t="n">
         <v>0.002209</v>
@@ -5467,12 +5652,12 @@
         <v>0.002142</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>313</v>
+        <v>328</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="53.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="6" t="s">
-        <v>314</v>
+        <v>329</v>
       </c>
       <c r="C9" s="31" t="n">
         <v>0.009059</v>
@@ -5481,17 +5666,17 @@
         <v>0.004507</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>315</v>
+        <v>330</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="14" t="s">
-        <v>316</v>
+        <v>331</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B12" s="32" t="s">
-        <v>317</v>
+        <v>332</v>
       </c>
       <c r="C12" s="32"/>
       <c r="D12" s="32"/>
@@ -5514,36 +5699,36 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="14" t="s">
-        <v>318</v>
+        <v>333</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="13" t="s">
-        <v>319</v>
+        <v>334</v>
       </c>
       <c r="C17" s="10" t="n">
         <f aca="false">3428-1340</f>
         <v>2088</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>320</v>
+        <v>335</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="13" t="s">
-        <v>321</v>
+        <v>336</v>
       </c>
       <c r="C18" s="10" t="n">
         <f aca="false">C17/0.05</f>
         <v>41760</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>322</v>
+        <v>337</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="13" t="s">
-        <v>323</v>
+        <v>338</v>
       </c>
       <c r="C19" s="9" t="n">
         <v>381944</v>
@@ -5552,19 +5737,19 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="13" t="s">
-        <v>324</v>
+        <v>339</v>
       </c>
       <c r="C20" s="10" t="n">
         <f aca="false">5027967+C17*288</f>
         <v>5629311</v>
       </c>
       <c r="F20" s="2" t="s">
-        <v>325</v>
+        <v>340</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="13" t="s">
-        <v>326</v>
+        <v>341</v>
       </c>
       <c r="C21" s="10" t="n">
         <f aca="false">C20/0.045709/288</f>
@@ -5574,7 +5759,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="13" t="s">
-        <v>327</v>
+        <v>342</v>
       </c>
       <c r="C22" s="9" t="n">
         <v>327778</v>
@@ -5583,31 +5768,31 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="13" t="s">
-        <v>328</v>
+        <v>343</v>
       </c>
       <c r="C23" s="15" t="n">
         <f aca="false">C22/C21-1</f>
         <v>-0.233488338914656</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>329</v>
+        <v>344</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="13" t="s">
-        <v>330</v>
+        <v>345</v>
       </c>
       <c r="C24" s="10" t="n">
         <f aca="false">(5904654-C17*360)/0.05/360</f>
         <v>286276.333333333</v>
       </c>
       <c r="F24" s="2" t="s">
-        <v>331</v>
+        <v>346</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B26" s="16" t="s">
-        <v>332</v>
+        <v>347</v>
       </c>
       <c r="C26" s="16"/>
       <c r="D26" s="16"/>
@@ -5652,12 +5837,12 @@
   <sheetData>
     <row r="2" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="1" t="s">
-        <v>333</v>
+        <v>348</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B4" s="14" t="s">
-        <v>334</v>
+        <v>349</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5671,7 +5856,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B6" s="6" t="s">
-        <v>335</v>
+        <v>350</v>
       </c>
       <c r="C6" s="8" t="n">
         <v>1130</v>
@@ -5682,7 +5867,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B7" s="6" t="s">
-        <v>336</v>
+        <v>351</v>
       </c>
       <c r="C7" s="8" t="n">
         <v>228</v>
@@ -5693,7 +5878,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B8" s="6" t="s">
-        <v>337</v>
+        <v>352</v>
       </c>
       <c r="C8" s="8" t="n">
         <v>507</v>
@@ -5704,7 +5889,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B9" s="6" t="s">
-        <v>338</v>
+        <v>353</v>
       </c>
       <c r="C9" s="8" t="n">
         <v>309</v>
@@ -5715,78 +5900,78 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="14" t="s">
-        <v>339</v>
+        <v>354</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="5" t="s">
-        <v>340</v>
+        <v>355</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>43</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>341</v>
+        <v>356</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="13" t="s">
-        <v>342</v>
+        <v>357</v>
       </c>
       <c r="C13" s="8" t="n">
         <v>552</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>343</v>
+        <v>358</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="13" t="s">
-        <v>344</v>
+        <v>359</v>
       </c>
       <c r="C14" s="8" t="n">
         <v>213</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>343</v>
+        <v>358</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="13" t="s">
-        <v>345</v>
+        <v>360</v>
       </c>
       <c r="C15" s="8" t="n">
         <v>212</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>346</v>
+        <v>361</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="13" t="s">
-        <v>347</v>
+        <v>362</v>
       </c>
       <c r="C16" s="8" t="n">
         <v>164</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>348</v>
+        <v>363</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="13" t="s">
-        <v>349</v>
+        <v>364</v>
       </c>
       <c r="C17" s="8" t="n">
         <v>72</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>346</v>
+        <v>361</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="17" t="s">
-        <v>350</v>
+        <v>365</v>
       </c>
       <c r="C18" s="33" t="n">
         <f aca="false">SUM(C13:C17)</f>
@@ -5795,12 +5980,12 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="14" t="s">
-        <v>351</v>
+        <v>366</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="5" t="s">
-        <v>340</v>
+        <v>355</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>43</v>
@@ -5808,7 +5993,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="13" t="s">
-        <v>352</v>
+        <v>367</v>
       </c>
       <c r="C22" s="8" t="n">
         <v>472</v>
@@ -5816,7 +6001,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="13" t="s">
-        <v>353</v>
+        <v>368</v>
       </c>
       <c r="C23" s="8" t="n">
         <v>390</v>
@@ -5824,7 +6009,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="13" t="s">
-        <v>354</v>
+        <v>369</v>
       </c>
       <c r="C24" s="8" t="n">
         <v>322</v>
@@ -5832,7 +6017,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="13" t="s">
-        <v>355</v>
+        <v>370</v>
       </c>
       <c r="C25" s="8" t="n">
         <v>301</v>
@@ -5840,7 +6025,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="13" t="s">
-        <v>356</v>
+        <v>371</v>
       </c>
       <c r="C26" s="8" t="n">
         <v>275</v>
@@ -5848,7 +6033,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="13" t="s">
-        <v>357</v>
+        <v>372</v>
       </c>
       <c r="C27" s="8" t="n">
         <v>270</v>
@@ -5856,7 +6041,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="13" t="s">
-        <v>358</v>
+        <v>373</v>
       </c>
       <c r="C28" s="8" t="n">
         <v>250</v>
@@ -5864,7 +6049,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="13" t="s">
-        <v>359</v>
+        <v>374</v>
       </c>
       <c r="C29" s="8" t="n">
         <v>200</v>
@@ -5872,7 +6057,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="13" t="s">
-        <v>360</v>
+        <v>375</v>
       </c>
       <c r="C30" s="8" t="n">
         <v>200</v>
@@ -5880,7 +6065,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B31" s="13" t="s">
-        <v>361</v>
+        <v>376</v>
       </c>
       <c r="C31" s="8" t="n">
         <v>162</v>
@@ -5888,7 +6073,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B32" s="13" t="s">
-        <v>362</v>
+        <v>377</v>
       </c>
       <c r="C32" s="8" t="n">
         <v>156</v>
@@ -5896,7 +6081,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B33" s="13" t="s">
-        <v>363</v>
+        <v>378</v>
       </c>
       <c r="C33" s="8" t="n">
         <v>138</v>
@@ -5904,7 +6089,7 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B34" s="13" t="s">
-        <v>364</v>
+        <v>379</v>
       </c>
       <c r="C34" s="8" t="n">
         <v>36</v>
@@ -5912,7 +6097,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B35" s="6" t="s">
-        <v>365</v>
+        <v>380</v>
       </c>
       <c r="C35" s="8" t="n">
         <v>256</v>
@@ -5920,7 +6105,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B36" s="17" t="s">
-        <v>366</v>
+        <v>381</v>
       </c>
       <c r="C36" s="33" t="n">
         <f aca="false">SUM(C22:C35)</f>
@@ -5929,7 +6114,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B38" s="16" t="s">
-        <v>367</v>
+        <v>382</v>
       </c>
       <c r="C38" s="16"/>
       <c r="D38" s="16"/>

</xml_diff>